<commit_message>
n8n board refresh 2026-09-07T17:42:22Z
</commit_message>
<xml_diff>
--- a/app/reports/LMT_research.xlsx
+++ b/app/reports/LMT_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-01 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-07 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.634</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>605.74</v>
+        <v>600.67</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>582.74</v>
+        <v>525.28</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.039</v>
+        <v>0.144</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.337</v>
+        <v>0.39</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.539</v>
+        <v>0.644</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04744999885559082</v>
+        <v>0.04783999919891357</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>230790741.5588427</v>
+        <v>230790760.6457509</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>582.74</v>
+        <v>525.28</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>134490996736</v>
+        <v>121229770752</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>21.5</v>
+        <v>19.38</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>15.62</v>
+        <v>14.25</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.96</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>105997787136</v>
+        <v>110288084992</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>24.334246</v>
+        <v>25.3766</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>16.764</v>
+        <v>17.403</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.883</v>
+        <v>5.084</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>170830577664</v>
+        <v>167756038144</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>77.46953600000001</v>
+        <v>76.34892000000001</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>-68.937</v>
+        <v>-67.877</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>2.127</v>
+        <v>2.094</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>159983812608</v>
+        <v>186993311744</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>33.56002</v>
+        <v>38.61526</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>23.175</v>
+        <v>26.353</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>4.217</v>
+        <v>4.729</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>103737040896</v>
+        <v>97235550208</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>23.365023</v>
+        <v>21.927397</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>16.392</v>
+        <v>15.413</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>1.982</v>
+        <v>1.864</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>77032267776</v>
+        <v>66433794048</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>9.344483</v>
+        <v>8.058824</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>12.114</v>
+        <v>10.869</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>2.709</v>
+        <v>2.431</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>51592622080</v>
+        <v>47754743808</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>28.014154</v>
+        <v>25.904043</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>31.838</v>
+        <v>29.715</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.315</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>77066346496</v>
+        <v>73159614464</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>17.243484</v>
+        <v>16.364157</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>12.655</v>
+        <v>12.116</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>2.141</v>
+        <v>2.049</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>123127144448</v>
+        <v>121332039680</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>35.967957</v>
+        <v>33.786945</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>24.136</v>
+        <v>22.877</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>6.301</v>
+        <v>6.027</v>
       </c>
     </row>
     <row r="15">

</xml_diff>